<commit_message>
integrated code scannerwith ML risk engineand updated generator
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -413,209 +413,489 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Test Case</t>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TC001 - [MAE ONLINE] Verify frontend allows transaction when RMBP=ON</t>
+          <t>TC_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Verify SST calculation applied correctly on Service Fee</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1. Initiate transfer
+2. Enter transfer amount
+3. Proceed to confirmation page
+4. Validate SST calculation</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SST must be calculated as per configured percentage and reflected correctly</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TC002 - [MAE ONLINE] Verify backend propagates SST when DCC=ON</t>
+          <t>TC_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Verify feature flag ON/OFF behavior</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1. Enable feature flag
+2. Perform transfer
+3. Disable feature flag
+4. Perform transfer again</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>System behavior must change according to feature flag state</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TC003 - [MAE ONLINE] Verify SST calculated correctly at configured percentage</t>
+          <t>TC_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Verify performance under high transaction load</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1. Simulate multiple concurrent transfers
+2. Monitor system response time</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>System should handle concurrent load without failure</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC004 - [MAE ONLINE] Verify total amount = principal + fee + SST</t>
+          <t>TC_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Verify transfer limit boundary validation</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1. Enter transfer amount equal to daily limit
+2. Submit transfer</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>System should allow transfer within configured limit</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TC005 - [MAE ONLINE] Verify ESB payload contains SST</t>
+          <t>TC_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Verify transfer exceeding daily limit is rejected</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1. Enter transfer amount exceeding daily limit
+2. Submit transfer</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>System must reject transaction exceeding configured limit</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TC006 - [MAE ONLINE] Verify CICS maps SST correctly</t>
+          <t>TC_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Verify fee rounding precision</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1. Enter amount with decimal value
+2. Proceed to confirmation</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Fee must be rounded correctly as per business rules</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TC007 - [MAE ONLINE] Verify core banking deducts total including SST</t>
+          <t>TC_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Verify SST applied to both service fee and agent fee</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1. Initiate transfer
+2. Review fee breakdown</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SST must be applied to all applicable fee components</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TC008 - [MAE ONLINE] Verify debit-credit reconciliation in core banking</t>
+          <t>TC_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Verify system error handling during transaction failure</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1. Simulate backend failure
+2. Submit transfer</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>System must show proper error message and prevent transaction completion</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TC009 - [MAE ONLINE] Validate API request includes SST field</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TC010 - [MAE ONLINE] Validate API response reflects updated fee structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TC011 - [MAE ONLINE] Verify CCPP reflects SST component correctly</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>TC012 - [MAE ONLINE] Verify RSA CQ/Deny/Review flow unaffected</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TC013 - [MAE OFFLINE] Verify frontend hides SST when RMBP=OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TC014 - [MAE OFFLINE] Verify backend suppresses SST when DCC=OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TC015 - [MAE OFFLINE] Verify no SST calculated</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TC016 - [MAE OFFLINE] Verify total amount excludes SST</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>TC017 - [MAE OFFLINE] Verify ESB payload excludes SST</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>TC018 - [MAE OFFLINE] Verify CICS does not map SST</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>TC019 - [MAE OFFLINE] Verify core banking deducts without SST</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TC020 - [MAE OFFLINE] Verify debit-credit reconciliation without SST</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TC021 - [MAE OFFLINE] Validate API request excludes SST field</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TC022 - [MAE OFFLINE] Validate API response excludes SST structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TC023 - Verify minimum transfer boundary amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>TC024 - Verify maximum transfer boundary amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>TC025 - Verify invalid amount scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>TC026 - Verify invalid currency scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>TC027 - Verify concurrent transactions handled correctly</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>TC028 - Verify performance under peak load</t>
+          <t>TC_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BAKONG</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Verify mandatory field validation</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>User logged into MAE and navigated to BAKONG module</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1. Leave mandatory fields blank
+2. Attempt to submit transfer</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>System must display validation message for mandatory fields</t>
         </is>
       </c>
     </row>

</xml_diff>